<commit_message>
Complete Week 03 Matplotlib visualization
</commit_message>
<xml_diff>
--- a/data/processed/cleaned_study_log.xlsx
+++ b/data/processed/cleaned_study_log.xlsx
@@ -518,7 +518,7 @@
         <v>90</v>
       </c>
       <c r="E4" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
@@ -596,7 +596,7 @@
         <v>60</v>
       </c>
       <c r="E7" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>

</xml_diff>